<commit_message>
Atualiza achados e automacoes de relatorios iGovTI
</commit_message>
<xml_diff>
--- a/02-Execucao/04-Matriz_Achados/mapa_rastreabilidade_achados.xlsx
+++ b/02-Execucao/04-Matriz_Achados/mapa_rastreabilidade_achados.xlsx
@@ -2324,7 +2324,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem governança técnica e controle de resultados</t>
+          <t>Fragilidades na governança técnica da fase preparatória das contratações de TIC</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem governança técnica e controle de resultados</t>
+          <t>Fragilidades na governança técnica da fase preparatória das contratações de TIC</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem governança técnica e controle de resultados</t>
+          <t>Fragilidades na governança técnica da fase preparatória das contratações de TIC</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem governança técnica e controle de resultados</t>
+          <t>Fragilidades na governança técnica da fase preparatória das contratações de TIC</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem governança técnica e controle de resultados</t>
+          <t>Fragilidades na governança técnica da fase preparatória das contratações de TIC</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">

</xml_diff>